<commit_message>
Auto HR search: updated contacts for 14 roles
</commit_message>
<xml_diff>
--- a/job-search/recommended_jobs.xlsx
+++ b/job-search/recommended_jobs.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="recommended_jobs" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HR_repository" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="recommended_jobs" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="HR_repository" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2364,7 +2364,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="65" customHeight="1">
+    <row r="2" ht="60" customHeight="1">
       <c r="A2" s="6" t="inlineStr">
         <is>
           <t>GPM - Subscription Renewals &amp; Revenue</t>
@@ -2387,27 +2387,19 @@
       </c>
       <c r="E2" s="6" t="inlineStr">
         <is>
-          <t>Priya Sharma</t>
+          <t>None Kavyanka Khanna</t>
         </is>
       </c>
       <c r="F2" s="6" t="inlineStr">
         <is>
-          <t>Tech Talent Partner</t>
-        </is>
-      </c>
-      <c r="G2" s="6" t="inlineStr">
-        <is>
-          <t>priya.sharma@jiohotstar.com</t>
-        </is>
-      </c>
-      <c r="H2" s="6" t="inlineStr">
-        <is>
-          <t>https://in.linkedin.com/in/priya-sharma-42636b193</t>
-        </is>
-      </c>
+          <t>Recruiter</t>
+        </is>
+      </c>
+      <c r="G2" s="6" t="inlineStr"/>
+      <c r="H2" s="6" t="inlineStr"/>
       <c r="I2" s="6" t="inlineStr">
         <is>
-          <t>LinkedIn search</t>
+          <t>Tavily Search</t>
         </is>
       </c>
       <c r="J2" s="7" t="inlineStr">
@@ -2417,11 +2409,11 @@
       </c>
       <c r="K2" s="6" t="inlineStr">
         <is>
-          <t>Email constructed from @jiohotstar.com first.last pattern (28% frequency). Connect on LinkedIn first.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="65" customHeight="1">
+          <t>No verified contact found — apply via company careers page or LinkedIn InMail.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="60" customHeight="1">
       <c r="A3" s="6" t="inlineStr">
         <is>
           <t>Sr PM - Growth / Membership</t>
@@ -2444,683 +2436,632 @@
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>Ritika Tyagi</t>
+          <t>Tal Prachi Rai</t>
         </is>
       </c>
       <c r="F3" s="6" t="inlineStr">
         <is>
+          <t>Recruiter</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>bluearmy911@gmail.com</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr"/>
+      <c r="I3" s="6" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="J3" s="8" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="K3" s="6" t="inlineStr">
+        <is>
+          <t>LinkedIn profile found. InMail recommended; email not verified.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="60" customHeight="1">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Sr PM - Trust &amp; Safety</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>PhonePe</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>Bangalore</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>Kirti Sharma</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
           <t>Talent Acquisition</t>
         </is>
       </c>
-      <c r="G3" s="6" t="inlineStr">
-        <is>
-          <t>ritika.tyagi@swiggy.in</t>
-        </is>
-      </c>
-      <c r="H3" s="6" t="inlineStr">
-        <is>
-          <t>https://in.linkedin.com/in/ritika-tyagi-579256146</t>
-        </is>
-      </c>
-      <c r="I3" s="6" t="inlineStr">
-        <is>
-          <t>LinkedIn + email pattern</t>
-        </is>
-      </c>
-      <c r="J3" s="8" t="inlineStr">
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>m@phonepe.com</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr"/>
+      <c r="I4" s="6" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="J4" s="8" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="K3" s="6" t="inlineStr">
-        <is>
-          <t>@swiggy.in first.last pattern confirmed at 93% frequency across employees.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="65" customHeight="1">
-      <c r="A4" s="6" t="inlineStr">
-        <is>
-          <t>Sr PM - Trust &amp; Safety</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="K4" s="6" t="inlineStr">
+        <is>
+          <t>LinkedIn profile found. InMail recommended; email not verified.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="60" customHeight="1">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>PM - Consumer Payments Growth</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>PhonePe</t>
         </is>
       </c>
-      <c r="C4" s="6" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="D4" s="6" t="inlineStr">
+      <c r="D5" s="6" t="inlineStr">
         <is>
           <t>Bangalore</t>
         </is>
       </c>
-      <c r="E4" s="6" t="inlineStr">
-        <is>
-          <t>Komal Sharma</t>
-        </is>
-      </c>
-      <c r="F4" s="6" t="inlineStr">
-        <is>
-          <t>Lead, Talent Acquisition</t>
-        </is>
-      </c>
-      <c r="G4" s="6" t="inlineStr">
-        <is>
-          <t>komal.sharma@phonepe.com</t>
-        </is>
-      </c>
-      <c r="H4" s="6" t="inlineStr">
-        <is>
-          <t>https://in.linkedin.com/in/komalsharma6</t>
-        </is>
-      </c>
-      <c r="I4" s="6" t="inlineStr">
-        <is>
-          <t>ContactOut / LinkedIn</t>
-        </is>
-      </c>
-      <c r="J4" s="8" t="inlineStr">
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>Kirti Sharma</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>Talent Acquisition</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>m@phonepe.com</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="inlineStr"/>
+      <c r="I5" s="6" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="J5" s="8" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="K4" s="6" t="inlineStr">
-        <is>
-          <t>Email format first.last@phonepe.com confirmed at 89.6%. ContactOut shows k***@phonepe.com.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="65" customHeight="1">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>PM - Consumer Payments Growth</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>PhonePe</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="K5" s="6" t="inlineStr">
+        <is>
+          <t>LinkedIn profile found. InMail recommended; email not verified.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="60" customHeight="1">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>PM / Sr PM</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>CRED</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="D5" s="6" t="inlineStr">
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>Bangalore</t>
         </is>
       </c>
-      <c r="E5" s="6" t="inlineStr">
-        <is>
-          <t>Komal Sharma</t>
-        </is>
-      </c>
-      <c r="F5" s="6" t="inlineStr">
-        <is>
-          <t>Lead, Talent Acquisition</t>
-        </is>
-      </c>
-      <c r="G5" s="6" t="inlineStr">
-        <is>
-          <t>komal.sharma@phonepe.com</t>
-        </is>
-      </c>
-      <c r="H5" s="6" t="inlineStr">
-        <is>
-          <t>https://in.linkedin.com/in/komalsharma6</t>
-        </is>
-      </c>
-      <c r="I5" s="6" t="inlineStr">
-        <is>
-          <t>ContactOut / LinkedIn</t>
-        </is>
-      </c>
-      <c r="J5" s="8" t="inlineStr">
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>years of experience driving</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>Talent Acquisition</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr"/>
+      <c r="H6" s="6" t="inlineStr"/>
+      <c r="I6" s="6" t="inlineStr">
+        <is>
+          <t>Tavily Search</t>
+        </is>
+      </c>
+      <c r="J6" s="7" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="K6" s="6" t="inlineStr">
+        <is>
+          <t>No verified contact found — apply via company careers page or LinkedIn InMail.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="60" customHeight="1">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>PM II - AI</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>Razorpay</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>Bangalore</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>Just your friendly Neighbourhood</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>Recruiter</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>prakhargupta1801@gmail.com</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="inlineStr"/>
+      <c r="I7" s="6" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="J7" s="8" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="K5" s="6" t="inlineStr">
-        <is>
-          <t>Same recruiter covers both PhonePe PM roles. Mention both roles in outreach.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="65" customHeight="1">
-      <c r="A6" s="6" t="inlineStr">
-        <is>
-          <t>PM / Sr PM</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>CRED</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="K7" s="6" t="inlineStr">
+        <is>
+          <t>LinkedIn profile found. InMail recommended; email not verified.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="60" customHeight="1">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>PM - Monetization &amp; Retention</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>Sarvam AI</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D8" s="6" t="inlineStr">
         <is>
           <t>Bangalore</t>
         </is>
       </c>
-      <c r="E6" s="6" t="inlineStr">
-        <is>
-          <t>Amanpreet Kaur</t>
-        </is>
-      </c>
-      <c r="F6" s="6" t="inlineStr">
-        <is>
-          <t>Talent &amp; Culture Leader</t>
-        </is>
-      </c>
-      <c r="G6" s="6" t="inlineStr">
-        <is>
-          <t>amankaur@cred.club</t>
-        </is>
-      </c>
-      <c r="H6" s="6" t="inlineStr">
-        <is>
-          <t>https://in.linkedin.com/in/hereamankaur</t>
-        </is>
-      </c>
-      <c r="I6" s="6" t="inlineStr">
-        <is>
-          <t>ZoomInfo / RocketReach</t>
-        </is>
-      </c>
-      <c r="J6" s="8" t="inlineStr">
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>transparency and the human touch to</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>Talent Acquisition</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>careers@sarvam.ai</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr"/>
+      <c r="I8" s="6" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="J8" s="8" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="K6" s="6" t="inlineStr">
-        <is>
-          <t>ZoomInfo confirms a***@cred.club. RocketReach shows amankaur@cred.club format. CRED email pattern first.last OR firstlast@cred.club (93%).</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="65" customHeight="1">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>PM II - AI</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>Razorpay</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="K8" s="6" t="inlineStr">
+        <is>
+          <t>LinkedIn profile found. InMail recommended; email not verified.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="60" customHeight="1">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>PM - Growth</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>Sarvam AI</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="D7" s="6" t="inlineStr">
+      <c r="D9" s="6" t="inlineStr">
         <is>
           <t>Bangalore</t>
         </is>
       </c>
-      <c r="E7" s="6" t="inlineStr">
-        <is>
-          <t>Sumit Premi</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>Senior Director &amp; Global Head, Talent Acquisition</t>
-        </is>
-      </c>
-      <c r="G7" s="6" t="inlineStr">
-        <is>
-          <t>sumit.premi@razorpay.com</t>
-        </is>
-      </c>
-      <c r="H7" s="6" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/sumit-premi-92349636/</t>
-        </is>
-      </c>
-      <c r="I7" s="6" t="inlineStr">
-        <is>
-          <t>ZoomInfo / LinkedIn</t>
-        </is>
-      </c>
-      <c r="J7" s="8" t="inlineStr">
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>transparency and the human touch to</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>Talent Acquisition</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>careers@sarvam.ai</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr"/>
+      <c r="I9" s="6" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="J9" s="8" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="K7" s="6" t="inlineStr">
-        <is>
-          <t>ZoomInfo confirms s***@razorpay.com. Email pattern first.last@razorpay.com at 92%. Active on LinkedIn — posted about AI hiring approach at Razorpay.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="65" customHeight="1">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>PM - Monetization &amp; Retention</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>Sarvam AI</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
+      <c r="K9" s="6" t="inlineStr">
+        <is>
+          <t>LinkedIn profile found. InMail recommended; email not verified.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="60" customHeight="1">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>Sr PM Tech - GenAI Compliance</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>Bangalore / Hyderabad</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>Recruiting Manager</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>Talent Acquisition</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>login@amazon.com</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/hollyrichardson1</t>
+        </is>
+      </c>
+      <c r="I10" s="6" t="inlineStr">
+        <is>
+          <t>LinkedIn + email</t>
+        </is>
+      </c>
+      <c r="J10" s="9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K10" s="6" t="inlineStr">
+        <is>
+          <t>Email and LinkedIn found. Verify before outreach.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="60" customHeight="1">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>Lead PM - Growth Platform</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>Uber</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
         <is>
           <t>Bangalore</t>
         </is>
       </c>
-      <c r="E8" s="6" t="inlineStr">
-        <is>
-          <t>Manikantha S</t>
-        </is>
-      </c>
-      <c r="F8" s="6" t="inlineStr">
-        <is>
-          <t>Head of Product (Hiring Manager)</t>
-        </is>
-      </c>
-      <c r="G8" s="6" t="inlineStr">
-        <is>
-          <t>manikantha@sarvam.ai</t>
-        </is>
-      </c>
-      <c r="H8" s="6" t="inlineStr">
-        <is>
-          <t>https://in.linkedin.com/in/manikantha</t>
-        </is>
-      </c>
-      <c r="I8" s="6" t="inlineStr">
-        <is>
-          <t>LinkedIn + email pattern</t>
-        </is>
-      </c>
-      <c r="J8" s="7" t="inlineStr">
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>to Linkedin</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>Recruiter</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr"/>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/devhall</t>
+        </is>
+      </c>
+      <c r="I11" s="6" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="J11" s="8" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="K11" s="6" t="inlineStr">
+        <is>
+          <t>LinkedIn profile found. InMail recommended; email not verified.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="60" customHeight="1">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>Staff PM - Viewer Experience</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>JioStar</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>Mumbai</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>None Kavyanka Khanna</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>Recruiter</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr"/>
+      <c r="H12" s="6" t="inlineStr"/>
+      <c r="I12" s="6" t="inlineStr">
+        <is>
+          <t>Tavily Search</t>
+        </is>
+      </c>
+      <c r="J12" s="7" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="K8" s="6" t="inlineStr">
-        <is>
-          <t>Small startup — no dedicated recruiter found. HM direct outreach preferred. Sarvam email pattern: first@sarvam.ai (92%). Apply directly via sarvam.ai/careers.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="65" customHeight="1">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>PM - Growth</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>Sarvam AI</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="inlineStr">
+      <c r="K12" s="6" t="inlineStr">
+        <is>
+          <t>No verified contact found — apply via company careers page or LinkedIn InMail.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="60" customHeight="1">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>Principal PM - AI Platform</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>Microsoft AI</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>Hyderabad</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>Jonathan Du Microsoft</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>Talent Acquisition</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr"/>
+      <c r="H13" s="6" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/brett-baumoel</t>
+        </is>
+      </c>
+      <c r="I13" s="6" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="J13" s="8" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="K13" s="6" t="inlineStr">
+        <is>
+          <t>LinkedIn profile found. InMail recommended; email not verified.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="60" customHeight="1">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>Group PM</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>Meesho</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
         <is>
           <t>Bangalore</t>
         </is>
       </c>
-      <c r="E9" s="6" t="inlineStr">
-        <is>
-          <t>Manikantha S</t>
-        </is>
-      </c>
-      <c r="F9" s="6" t="inlineStr">
-        <is>
-          <t>Head of Product (Hiring Manager)</t>
-        </is>
-      </c>
-      <c r="G9" s="6" t="inlineStr">
-        <is>
-          <t>manikantha@sarvam.ai</t>
-        </is>
-      </c>
-      <c r="H9" s="6" t="inlineStr">
-        <is>
-          <t>https://in.linkedin.com/in/manikantha</t>
-        </is>
-      </c>
-      <c r="I9" s="6" t="inlineStr">
-        <is>
-          <t>LinkedIn + email pattern</t>
-        </is>
-      </c>
-      <c r="J9" s="7" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="K9" s="6" t="inlineStr">
-        <is>
-          <t>Same HM for both Sarvam PM roles. Startup context — LinkedIn DM + job portal application recommended.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="65" customHeight="1">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>Sr PM Tech - GenAI Compliance</t>
-        </is>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>HR Recruiter at Meesho Sonal Singh
+HR</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>Recruiter</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>mei.ragavendiran@meesho.com</t>
+        </is>
+      </c>
+      <c r="H14" s="6" t="inlineStr"/>
+      <c r="I14" s="6" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="J14" s="8" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="K14" s="6" t="inlineStr">
+        <is>
+          <t>LinkedIn profile found. InMail recommended; email not verified.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="60" customHeight="1">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>Staff PM</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>Freshworks</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="D10" s="6" t="inlineStr">
-        <is>
-          <t>Bangalore / Hyderabad</t>
-        </is>
-      </c>
-      <c r="E10" s="6" t="inlineStr">
-        <is>
-          <t>Priyanka Pathak</t>
-        </is>
-      </c>
-      <c r="F10" s="6" t="inlineStr">
-        <is>
-          <t>Talent Acquisition Recruiter</t>
-        </is>
-      </c>
-      <c r="G10" s="6" t="inlineStr">
-        <is>
-          <t>priyanka.pathak@amazon.com</t>
-        </is>
-      </c>
-      <c r="H10" s="6" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/priyankapathak03/</t>
-        </is>
-      </c>
-      <c r="I10" s="6" t="inlineStr">
-        <is>
-          <t>LinkedIn search</t>
-        </is>
-      </c>
-      <c r="J10" s="7" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="K10" s="6" t="inlineStr">
-        <is>
-          <t>Amazon has complex email formats; first.last@amazon.com is most common. Apply via amazon.jobs portal primarily. LinkedIn InMail more reliable for Amazon.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="65" customHeight="1">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>Lead PM - Growth Platform</t>
-        </is>
-      </c>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t>Uber</t>
-        </is>
-      </c>
-      <c r="C11" s="6" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="D11" s="6" t="inlineStr">
-        <is>
-          <t>Bangalore</t>
-        </is>
-      </c>
-      <c r="E11" s="6" t="inlineStr">
-        <is>
-          <t>Urvi Chauhan</t>
-        </is>
-      </c>
-      <c r="F11" s="6" t="inlineStr">
-        <is>
-          <t>Senior Recruiter, India &amp; South Asia</t>
-        </is>
-      </c>
-      <c r="G11" s="6" t="inlineStr">
-        <is>
-          <t>urvi.chauhan@uber.com</t>
-        </is>
-      </c>
-      <c r="H11" s="6" t="inlineStr">
-        <is>
-          <t>https://in.linkedin.com/in/urvichauhan</t>
-        </is>
-      </c>
-      <c r="I11" s="6" t="inlineStr">
-        <is>
-          <t>LinkedIn search</t>
-        </is>
-      </c>
-      <c r="J11" s="7" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="K11" s="6" t="inlineStr">
-        <is>
-          <t>Email constructed from standard Uber first.last@uber.com pattern. LinkedIn outreach preferred — Urvi is active on LinkedIn.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="65" customHeight="1">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>Staff PM - Viewer Experience</t>
-        </is>
-      </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>JioStar</t>
-        </is>
-      </c>
-      <c r="C12" s="6" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="D12" s="6" t="inlineStr">
-        <is>
-          <t>Mumbai</t>
-        </is>
-      </c>
-      <c r="E12" s="6" t="inlineStr">
-        <is>
-          <t>Priya Sharma</t>
-        </is>
-      </c>
-      <c r="F12" s="6" t="inlineStr">
-        <is>
-          <t>Tech Talent Partner</t>
-        </is>
-      </c>
-      <c r="G12" s="6" t="inlineStr">
-        <is>
-          <t>priya.sharma@jiohotstar.com</t>
-        </is>
-      </c>
-      <c r="H12" s="6" t="inlineStr">
-        <is>
-          <t>https://in.linkedin.com/in/priya-sharma-42636b193</t>
-        </is>
-      </c>
-      <c r="I12" s="6" t="inlineStr">
-        <is>
-          <t>LinkedIn search</t>
-        </is>
-      </c>
-      <c r="J12" s="7" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="K12" s="6" t="inlineStr">
-        <is>
-          <t>Same recruiter as JioStar GPM role. Mention both roles (GPM + Staff PM) in one outreach to avoid duplicate contacts.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="65" customHeight="1">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>Principal PM - AI Platform</t>
-        </is>
-      </c>
-      <c r="B13" s="6" t="inlineStr">
-        <is>
-          <t>Microsoft AI</t>
-        </is>
-      </c>
-      <c r="C13" s="6" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="D13" s="6" t="inlineStr">
-        <is>
-          <t>Hyderabad</t>
-        </is>
-      </c>
-      <c r="E13" s="6" t="inlineStr">
-        <is>
-          <t>Ramya H R</t>
-        </is>
-      </c>
-      <c r="F13" s="6" t="inlineStr">
-        <is>
-          <t>Lead Talent Acquisition Specialist</t>
-        </is>
-      </c>
-      <c r="G13" s="6" t="inlineStr">
-        <is>
-          <t>ramya.hr@microsoft.com</t>
-        </is>
-      </c>
-      <c r="H13" s="6" t="inlineStr">
-        <is>
-          <t>https://in.linkedin.com/in/ramya-h-r-859155a</t>
-        </is>
-      </c>
-      <c r="I13" s="6" t="inlineStr">
-        <is>
-          <t>LinkedIn search</t>
-        </is>
-      </c>
-      <c r="J13" s="7" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="K13" s="6" t="inlineStr">
-        <is>
-          <t>Email constructed from first.last@microsoft.com pattern. Microsoft roles best applied via careers.microsoft.com. LinkedIn InMail recommended over cold email.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="65" customHeight="1">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>Group PM</t>
-        </is>
-      </c>
-      <c r="B14" s="6" t="inlineStr">
-        <is>
-          <t>Meesho</t>
-        </is>
-      </c>
-      <c r="C14" s="6" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="D14" s="6" t="inlineStr">
-        <is>
-          <t>Bangalore</t>
-        </is>
-      </c>
-      <c r="E14" s="6" t="inlineStr">
-        <is>
-          <t>SriKartik Sayana</t>
-        </is>
-      </c>
-      <c r="F14" s="6" t="inlineStr">
-        <is>
-          <t>Director, Talent Acquisition</t>
-        </is>
-      </c>
-      <c r="G14" s="6" t="inlineStr">
-        <is>
-          <t>srikartik.sayana@meesho.com</t>
-        </is>
-      </c>
-      <c r="H14" s="6" t="inlineStr">
-        <is>
-          <t>https://in.linkedin.com/in/srikartiksayana</t>
-        </is>
-      </c>
-      <c r="I14" s="6" t="inlineStr">
-        <is>
-          <t>ContactOut / ZoomInfo</t>
-        </is>
-      </c>
-      <c r="J14" s="9" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="K14" s="6" t="inlineStr">
-        <is>
-          <t>Email confirmed by multiple sources (ContactOut, ZoomInfo, Weekday.works). Apply via meesho.io/jobs + follow up with direct email.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="65" customHeight="1">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>Staff PM</t>
-        </is>
-      </c>
-      <c r="B15" s="6" t="inlineStr">
-        <is>
-          <t>Freshworks</t>
-        </is>
-      </c>
-      <c r="C15" s="6" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
           <t>Chennai</t>
@@ -3128,37 +3069,34 @@
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>Sasikumar S</t>
+          <t>About
+Senior</t>
         </is>
       </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
-          <t>Lead Talent Acquisition</t>
-        </is>
-      </c>
-      <c r="G15" s="6" t="inlineStr">
-        <is>
-          <t>sasikumar.s@freshworks.com</t>
-        </is>
-      </c>
+          <t>Recruiter</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="inlineStr"/>
       <c r="H15" s="6" t="inlineStr">
         <is>
-          <t>https://in.linkedin.com/in/sasikumar-recruiter</t>
+          <t>https://www.linkedin.com/in/alli-wojchik</t>
         </is>
       </c>
       <c r="I15" s="6" t="inlineStr">
         <is>
-          <t>LinkedIn / RocketReach</t>
-        </is>
-      </c>
-      <c r="J15" s="7" t="inlineStr">
-        <is>
-          <t>Low</t>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="J15" s="8" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="K15" s="6" t="inlineStr">
         <is>
-          <t>RocketReach shows s***@freshworks.com. Exact format for single-word last name unclear — try sasikumar@freshworks.com if first attempt bounces. Apply via freshworks.com/careers.</t>
+          <t>LinkedIn profile found. InMail recommended; email not verified.</t>
         </is>
       </c>
     </row>

</xml_diff>